<commit_message>
Add user sheet management features and update various components
</commit_message>
<xml_diff>
--- a/data/raw/건물토지매매.xlsx
+++ b/data/raw/건물토지매매.xlsx
@@ -10690,7 +10690,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -10776,7 +10776,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">

</xml_diff>

<commit_message>
Update project files and add new features
</commit_message>
<xml_diff>
--- a/data/raw/건물토지매매.xlsx
+++ b/data/raw/건물토지매매.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X154"/>
+  <dimension ref="A1:X155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -616,7 +616,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -714,7 +714,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2754,7 +2754,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4252,7 +4252,7 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -5176,7 +5176,7 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -7032,7 +7032,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -7600,7 +7600,7 @@
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8074,12 +8074,12 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>19000</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>1180</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -8104,12 +8104,12 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.33%</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>입55억, 2층3000/200,3층4000/150,4층2000/160,</t>
+          <t>입55억, 1층3000/280, 2층3000/200,3층4000/150,4층5000/140,5층6층2000/160, 관리비1-4층12만 5-6층 10만</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -8447,7 +8447,7 @@
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -9457,7 +9457,7 @@
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -9555,7 +9555,7 @@
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -11646,11 +11646,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>ㅁ</t>
-        </is>
-      </c>
+      <c r="A119" t="inlineStr"/>
       <c r="B119" t="inlineStr">
         <is>
           <t>250117</t>
@@ -11720,7 +11716,11 @@
       <c r="X119" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>ㅁ</t>
+        </is>
+      </c>
       <c r="B120" t="inlineStr">
         <is>
           <t>250120</t>
@@ -12374,11 +12374,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>ㅁ</t>
-        </is>
-      </c>
+      <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr">
         <is>
           <t>250208</t>
@@ -12435,7 +12431,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -12464,7 +12460,11 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>ㅁ</t>
+        </is>
+      </c>
       <c r="B129" t="inlineStr">
         <is>
           <t>250303</t>
@@ -12651,7 +12651,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
@@ -14233,61 +14233,85 @@
     </row>
     <row r="150">
       <c r="A150" t="inlineStr"/>
-      <c r="B150" t="inlineStr"/>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>250908</t>
+        </is>
+      </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>청천동</t>
+          <t>청라동</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>9-1</t>
+          <t>142-3</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
-      <c r="M150" t="inlineStr"/>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>54500</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>444</t>
+        </is>
+      </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>230,000</t>
+          <t>185,000</t>
         </is>
       </c>
       <c r="O150" t="inlineStr"/>
-      <c r="P150" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="Q150" t="inlineStr">
-        <is>
-          <t>3.50%</t>
-        </is>
-      </c>
-      <c r="R150" t="inlineStr"/>
+      <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>4.08%</t>
+        </is>
+      </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>지하50, 1층 커피숍3000/250, 2층1000/150, 3층1000/80, 4층 주택 전세1억 원룸2개 월세50가능</t>
-        </is>
-      </c>
-      <c r="T150" t="inlineStr"/>
-      <c r="U150" t="inlineStr"/>
-      <c r="V150" t="inlineStr"/>
-      <c r="W150" t="inlineStr"/>
-      <c r="X150" t="inlineStr"/>
+          <t xml:space="preserve">1층 1호 1000/90, 2호 1000/84, 3호~5호 각 1000/90, 2층 1호 전14000 2호 전18000 각 방3화2 3층전부+4층다락 전 16500 / 다락 방2화2, 몇 안되는 엘베있는 건물. 3층 천장쪽 판넬로 막음. 위반여지있음. </t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>남</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>생</t>
+        </is>
+      </c>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>소유주</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>본인</t>
+        </is>
+      </c>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>010-2588-6734</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr"/>
@@ -14327,7 +14351,7 @@
       <c r="O151" t="inlineStr"/>
       <c r="P151" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="Q151" t="inlineStr">
@@ -14352,16 +14376,20 @@
       <c r="B152" t="inlineStr"/>
       <c r="C152" t="inlineStr">
         <is>
-          <t>가좌동</t>
+          <t>청천동</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>212-4</t>
+          <t>9-1</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="G152" t="inlineStr">
         <is>
           <t>4</t>
@@ -14375,7 +14403,7 @@
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="inlineStr">
         <is>
-          <t>140,000</t>
+          <t>230,000</t>
         </is>
       </c>
       <c r="O152" t="inlineStr"/>
@@ -14392,86 +14420,90 @@
       <c r="R152" t="inlineStr"/>
       <c r="S152" t="inlineStr">
         <is>
-          <t>130000까지</t>
-        </is>
-      </c>
-      <c r="T152" t="inlineStr">
-        <is>
-          <t>오</t>
-        </is>
-      </c>
-      <c r="U152" t="inlineStr">
-        <is>
-          <t>생</t>
-        </is>
-      </c>
+          <t>지하50, 1층 커피숍3000/250, 2층1000/150, 3층1000/80, 4층 주택 전세1억 원룸2개 월세50가능</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr"/>
       <c r="V152" t="inlineStr"/>
-      <c r="W152" t="inlineStr">
-        <is>
-          <t>임대인</t>
-        </is>
-      </c>
-      <c r="X152" t="inlineStr">
-        <is>
-          <t>010-4036-8150</t>
-        </is>
-      </c>
+      <c r="W152" t="inlineStr"/>
+      <c r="X152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr"/>
       <c r="B153" t="inlineStr"/>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>가좌동</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>212-4</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>450</t>
-        </is>
-      </c>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr"/>
       <c r="N153" t="inlineStr">
         <is>
           <t>140,000</t>
         </is>
       </c>
       <c r="O153" t="inlineStr"/>
-      <c r="P153" t="inlineStr"/>
-      <c r="Q153" t="inlineStr"/>
-      <c r="R153" t="inlineStr">
-        <is>
-          <t>4.03%</t>
-        </is>
-      </c>
-      <c r="S153" t="inlineStr"/>
-      <c r="T153" t="inlineStr"/>
-      <c r="U153" t="inlineStr"/>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>3.50%</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>130000까지</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>오</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>생</t>
+        </is>
+      </c>
       <c r="V153" t="inlineStr"/>
-      <c r="W153" t="inlineStr"/>
-      <c r="X153" t="inlineStr"/>
+      <c r="W153" t="inlineStr">
+        <is>
+          <t>임대인</t>
+        </is>
+      </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>010-4036-8150</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr"/>
       <c r="B154" t="inlineStr"/>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>부평동</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>633-8</t>
-        </is>
-      </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr"/>
@@ -14479,35 +14511,85 @@
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr"/>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>130,000</t>
+          <t>140,000</t>
         </is>
       </c>
       <c r="O154" t="inlineStr"/>
-      <c r="P154" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q154" t="inlineStr">
-        <is>
-          <t>3.50%</t>
-        </is>
-      </c>
-      <c r="R154" t="inlineStr"/>
-      <c r="S154" t="inlineStr">
-        <is>
-          <t>미래부동산 매물 손님 연력 해달라고 함</t>
-        </is>
-      </c>
+      <c r="P154" t="inlineStr"/>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>4.03%</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr"/>
       <c r="T154" t="inlineStr"/>
       <c r="U154" t="inlineStr"/>
       <c r="V154" t="inlineStr"/>
       <c r="W154" t="inlineStr"/>
-      <c r="X154" t="inlineStr">
+      <c r="X154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr"/>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>부평동</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>633-8</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr"/>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>130,000</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr"/>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>3.50%</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>미래부동산 매물 손님 연력 해달라고 함</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr"/>
+      <c r="U155" t="inlineStr"/>
+      <c r="V155" t="inlineStr"/>
+      <c r="W155" t="inlineStr"/>
+      <c r="X155" t="inlineStr">
         <is>
           <t>010-2355-6511</t>
         </is>

</xml_diff>